<commit_message>
Update metadata to Health-RI v2.0.3
Upgrade to Health-RI v2.0.3 specification and regenerate property documentation.

Changes include:
- Updated Excel metadata specification from v2.0.2 to v2.0.3
- Corrected type definitions (e.g., xsd:string → rdfs:Literal)
- Updated cardinalities for dataset requirement (0..n → 1..n)
- Enhanced creator and contact point descriptions with clarifications
- Standardized contact point language across all properties
- Fixed formatting and URL protocols
- Improved documentation with additional guidance and examples
</commit_message>
<xml_diff>
--- a/src/excel/HealthRI_v2.0.2.xlsx
+++ b/src/excel/HealthRI_v2.0.2.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D452F6-957B-427A-8247-D60DE431818C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11604" windowHeight="13776" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -4101,32 +4101,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -4140,8 +4137,11 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -9796,40 +9796,40 @@
       </c>
     </row>
     <row r="6" spans="1:21" ht="28.8">
-      <c r="A6" s="231" t="s">
+      <c r="A6" s="230" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="232" t="s">
+      <c r="B6" s="231" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="231" t="s">
+      <c r="C6" s="230" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="234" t="s">
+      <c r="D6" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E6" s="233" t="s">
+      <c r="E6" s="232" t="s">
         <v>98</v>
       </c>
-      <c r="F6" s="230" t="s">
+      <c r="F6" s="229" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="230" t="s">
+      <c r="G6" s="229" t="s">
         <v>99</v>
       </c>
-      <c r="H6" s="230" t="s">
+      <c r="H6" s="229" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="228" t="s">
+      <c r="I6" s="233" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="225" t="s">
+      <c r="J6" s="222" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="229" t="s">
+      <c r="K6" s="234" t="s">
         <v>456</v>
       </c>
-      <c r="L6" s="228"/>
+      <c r="L6" s="233"/>
       <c r="M6" s="32" t="s">
         <v>703</v>
       </c>
@@ -9847,68 +9847,68 @@
       </c>
     </row>
     <row r="7" spans="1:21" ht="28.8">
-      <c r="A7" s="231"/>
-      <c r="B7" s="232"/>
-      <c r="C7" s="231"/>
-      <c r="D7" s="234" t="s">
+      <c r="A7" s="230"/>
+      <c r="B7" s="231"/>
+      <c r="C7" s="230"/>
+      <c r="D7" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E7" s="233"/>
-      <c r="F7" s="230"/>
-      <c r="G7" s="230"/>
-      <c r="H7" s="230"/>
-      <c r="I7" s="228"/>
-      <c r="J7" s="225"/>
-      <c r="K7" s="229"/>
-      <c r="L7" s="228"/>
+      <c r="E7" s="232"/>
+      <c r="F7" s="229"/>
+      <c r="G7" s="229"/>
+      <c r="H7" s="229"/>
+      <c r="I7" s="233"/>
+      <c r="J7" s="222"/>
+      <c r="K7" s="234"/>
+      <c r="L7" s="233"/>
     </row>
     <row r="8" spans="1:21" ht="28.8">
-      <c r="A8" s="231"/>
-      <c r="B8" s="232"/>
-      <c r="C8" s="231"/>
-      <c r="D8" s="234" t="s">
+      <c r="A8" s="230"/>
+      <c r="B8" s="231"/>
+      <c r="C8" s="230"/>
+      <c r="D8" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E8" s="233"/>
-      <c r="F8" s="230"/>
-      <c r="G8" s="230"/>
-      <c r="H8" s="230"/>
-      <c r="I8" s="228"/>
-      <c r="J8" s="225"/>
-      <c r="K8" s="229"/>
-      <c r="L8" s="228"/>
+      <c r="E8" s="232"/>
+      <c r="F8" s="229"/>
+      <c r="G8" s="229"/>
+      <c r="H8" s="229"/>
+      <c r="I8" s="233"/>
+      <c r="J8" s="222"/>
+      <c r="K8" s="234"/>
+      <c r="L8" s="233"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="231"/>
-      <c r="B9" s="232"/>
-      <c r="C9" s="231"/>
-      <c r="D9" s="234" t="s">
+      <c r="A9" s="230"/>
+      <c r="B9" s="231"/>
+      <c r="C9" s="230"/>
+      <c r="D9" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E9" s="233"/>
-      <c r="F9" s="230"/>
-      <c r="G9" s="230"/>
-      <c r="H9" s="230"/>
-      <c r="I9" s="228"/>
-      <c r="J9" s="225"/>
-      <c r="K9" s="229"/>
-      <c r="L9" s="228"/>
+      <c r="E9" s="232"/>
+      <c r="F9" s="229"/>
+      <c r="G9" s="229"/>
+      <c r="H9" s="229"/>
+      <c r="I9" s="233"/>
+      <c r="J9" s="222"/>
+      <c r="K9" s="234"/>
+      <c r="L9" s="233"/>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="231"/>
-      <c r="B10" s="232"/>
-      <c r="C10" s="231"/>
-      <c r="D10" s="234" t="s">
+      <c r="A10" s="230"/>
+      <c r="B10" s="231"/>
+      <c r="C10" s="230"/>
+      <c r="D10" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E10" s="233"/>
-      <c r="F10" s="230"/>
-      <c r="G10" s="230"/>
-      <c r="H10" s="230"/>
-      <c r="I10" s="228"/>
-      <c r="J10" s="225"/>
-      <c r="K10" s="229"/>
-      <c r="L10" s="228"/>
+      <c r="E10" s="232"/>
+      <c r="F10" s="229"/>
+      <c r="G10" s="229"/>
+      <c r="H10" s="229"/>
+      <c r="I10" s="233"/>
+      <c r="J10" s="222"/>
+      <c r="K10" s="234"/>
+      <c r="L10" s="233"/>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="121" t="s">
@@ -10303,17 +10303,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -11281,7 +11281,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="57.6">
+    <row r="18" spans="1:21" ht="43.2">
       <c r="A18" s="121" t="s">
         <v>155</v>
       </c>
@@ -16172,74 +16172,74 @@
       <c r="L13" s="129"/>
     </row>
     <row r="14" spans="1:20">
-      <c r="A14" s="222"/>
-      <c r="B14" s="223"/>
-      <c r="C14" s="222"/>
+      <c r="A14" s="224"/>
+      <c r="B14" s="228"/>
+      <c r="C14" s="224"/>
       <c r="D14" s="151"/>
-      <c r="E14" s="224"/>
-      <c r="F14" s="221"/>
-      <c r="G14" s="221"/>
-      <c r="H14" s="221"/>
-      <c r="I14" s="225"/>
-      <c r="J14" s="225"/>
-      <c r="K14" s="226"/>
-      <c r="L14" s="225"/>
+      <c r="E14" s="226"/>
+      <c r="F14" s="223"/>
+      <c r="G14" s="223"/>
+      <c r="H14" s="223"/>
+      <c r="I14" s="222"/>
+      <c r="J14" s="222"/>
+      <c r="K14" s="227"/>
+      <c r="L14" s="222"/>
     </row>
     <row r="15" spans="1:20">
-      <c r="A15" s="222"/>
-      <c r="B15" s="223"/>
-      <c r="C15" s="222"/>
+      <c r="A15" s="224"/>
+      <c r="B15" s="228"/>
+      <c r="C15" s="224"/>
       <c r="D15" s="152"/>
-      <c r="E15" s="224"/>
-      <c r="F15" s="221"/>
-      <c r="G15" s="221"/>
-      <c r="H15" s="221"/>
-      <c r="I15" s="225"/>
-      <c r="J15" s="225"/>
-      <c r="K15" s="226"/>
-      <c r="L15" s="225"/>
+      <c r="E15" s="226"/>
+      <c r="F15" s="223"/>
+      <c r="G15" s="223"/>
+      <c r="H15" s="223"/>
+      <c r="I15" s="222"/>
+      <c r="J15" s="222"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="222"/>
     </row>
     <row r="16" spans="1:20">
-      <c r="A16" s="222"/>
-      <c r="B16" s="223"/>
-      <c r="C16" s="222"/>
+      <c r="A16" s="224"/>
+      <c r="B16" s="228"/>
+      <c r="C16" s="224"/>
       <c r="D16" s="152"/>
-      <c r="E16" s="224"/>
-      <c r="F16" s="221"/>
-      <c r="G16" s="221"/>
-      <c r="H16" s="221"/>
-      <c r="I16" s="225"/>
-      <c r="J16" s="225"/>
-      <c r="K16" s="226"/>
-      <c r="L16" s="225"/>
+      <c r="E16" s="226"/>
+      <c r="F16" s="223"/>
+      <c r="G16" s="223"/>
+      <c r="H16" s="223"/>
+      <c r="I16" s="222"/>
+      <c r="J16" s="222"/>
+      <c r="K16" s="227"/>
+      <c r="L16" s="222"/>
     </row>
     <row r="17" spans="1:12">
-      <c r="A17" s="222"/>
-      <c r="B17" s="223"/>
-      <c r="C17" s="222"/>
+      <c r="A17" s="224"/>
+      <c r="B17" s="228"/>
+      <c r="C17" s="224"/>
       <c r="D17" s="152"/>
-      <c r="E17" s="224"/>
-      <c r="F17" s="221"/>
-      <c r="G17" s="221"/>
-      <c r="H17" s="221"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="225"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="225"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="223"/>
+      <c r="G17" s="223"/>
+      <c r="H17" s="223"/>
+      <c r="I17" s="222"/>
+      <c r="J17" s="222"/>
+      <c r="K17" s="227"/>
+      <c r="L17" s="222"/>
     </row>
     <row r="18" spans="1:12">
-      <c r="A18" s="222"/>
-      <c r="B18" s="223"/>
-      <c r="C18" s="222"/>
+      <c r="A18" s="224"/>
+      <c r="B18" s="228"/>
+      <c r="C18" s="224"/>
       <c r="D18" s="152"/>
-      <c r="E18" s="224"/>
-      <c r="F18" s="221"/>
-      <c r="G18" s="221"/>
-      <c r="H18" s="221"/>
-      <c r="I18" s="225"/>
-      <c r="J18" s="225"/>
-      <c r="K18" s="226"/>
-      <c r="L18" s="225"/>
+      <c r="E18" s="226"/>
+      <c r="F18" s="223"/>
+      <c r="G18" s="223"/>
+      <c r="H18" s="223"/>
+      <c r="I18" s="222"/>
+      <c r="J18" s="222"/>
+      <c r="K18" s="227"/>
+      <c r="L18" s="222"/>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="125"/>
@@ -16747,17 +16747,17 @@
   </sheetData>
   <autoFilter ref="A1:J53" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="11">
-    <mergeCell ref="H14:H18"/>
-    <mergeCell ref="I14:I18"/>
-    <mergeCell ref="J14:J18"/>
-    <mergeCell ref="K14:K18"/>
-    <mergeCell ref="L14:L18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="A14:A18"/>
     <mergeCell ref="B14:B18"/>
     <mergeCell ref="C14:C18"/>
     <mergeCell ref="E14:E18"/>
     <mergeCell ref="F14:F18"/>
+    <mergeCell ref="H14:H18"/>
+    <mergeCell ref="I14:I18"/>
+    <mergeCell ref="J14:J18"/>
+    <mergeCell ref="K14:K18"/>
+    <mergeCell ref="L14:L18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="204" priority="8" operator="equal">
@@ -17555,38 +17555,38 @@
       </c>
     </row>
     <row r="14" spans="1:21" ht="43.2">
-      <c r="A14" s="222" t="s">
+      <c r="A14" s="224" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="223" t="s">
+      <c r="B14" s="228" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="222" t="s">
+      <c r="C14" s="224" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="234" t="s">
+      <c r="D14" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E14" s="224" t="s">
+      <c r="E14" s="226" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="221" t="s">
+      <c r="F14" s="223" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="221" t="s">
+      <c r="G14" s="223" t="s">
         <v>99</v>
       </c>
-      <c r="H14" s="221" t="s">
+      <c r="H14" s="223" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="225" t="s">
+      <c r="I14" s="222" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="225" t="s">
+      <c r="J14" s="222" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="226"/>
-      <c r="L14" s="225"/>
+      <c r="K14" s="227"/>
+      <c r="L14" s="222"/>
       <c r="M14" s="32" t="s">
         <v>703</v>
       </c>
@@ -17604,68 +17604,68 @@
       </c>
     </row>
     <row r="15" spans="1:21" ht="43.2">
-      <c r="A15" s="222"/>
-      <c r="B15" s="223"/>
-      <c r="C15" s="222"/>
-      <c r="D15" s="234" t="s">
+      <c r="A15" s="224"/>
+      <c r="B15" s="228"/>
+      <c r="C15" s="224"/>
+      <c r="D15" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E15" s="224"/>
-      <c r="F15" s="221"/>
-      <c r="G15" s="221"/>
-      <c r="H15" s="221"/>
-      <c r="I15" s="225"/>
-      <c r="J15" s="225"/>
-      <c r="K15" s="226"/>
-      <c r="L15" s="225"/>
+      <c r="E15" s="226"/>
+      <c r="F15" s="223"/>
+      <c r="G15" s="223"/>
+      <c r="H15" s="223"/>
+      <c r="I15" s="222"/>
+      <c r="J15" s="222"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="222"/>
     </row>
     <row r="16" spans="1:21" ht="28.8">
-      <c r="A16" s="222"/>
-      <c r="B16" s="223"/>
-      <c r="C16" s="222"/>
-      <c r="D16" s="234" t="s">
+      <c r="A16" s="224"/>
+      <c r="B16" s="228"/>
+      <c r="C16" s="224"/>
+      <c r="D16" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E16" s="224"/>
-      <c r="F16" s="221"/>
-      <c r="G16" s="221"/>
-      <c r="H16" s="221"/>
-      <c r="I16" s="225"/>
-      <c r="J16" s="225"/>
-      <c r="K16" s="226"/>
-      <c r="L16" s="225"/>
+      <c r="E16" s="226"/>
+      <c r="F16" s="223"/>
+      <c r="G16" s="223"/>
+      <c r="H16" s="223"/>
+      <c r="I16" s="222"/>
+      <c r="J16" s="222"/>
+      <c r="K16" s="227"/>
+      <c r="L16" s="222"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="222"/>
-      <c r="B17" s="223"/>
-      <c r="C17" s="222"/>
-      <c r="D17" s="234" t="s">
+      <c r="A17" s="224"/>
+      <c r="B17" s="228"/>
+      <c r="C17" s="224"/>
+      <c r="D17" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E17" s="224"/>
-      <c r="F17" s="221"/>
-      <c r="G17" s="221"/>
-      <c r="H17" s="221"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="225"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="225"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="223"/>
+      <c r="G17" s="223"/>
+      <c r="H17" s="223"/>
+      <c r="I17" s="222"/>
+      <c r="J17" s="222"/>
+      <c r="K17" s="227"/>
+      <c r="L17" s="222"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="222"/>
-      <c r="B18" s="223"/>
-      <c r="C18" s="222"/>
-      <c r="D18" s="234" t="s">
+      <c r="A18" s="224"/>
+      <c r="B18" s="228"/>
+      <c r="C18" s="224"/>
+      <c r="D18" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E18" s="224"/>
-      <c r="F18" s="221"/>
-      <c r="G18" s="221"/>
-      <c r="H18" s="221"/>
-      <c r="I18" s="225"/>
-      <c r="J18" s="225"/>
-      <c r="K18" s="226"/>
-      <c r="L18" s="225"/>
+      <c r="E18" s="226"/>
+      <c r="F18" s="223"/>
+      <c r="G18" s="223"/>
+      <c r="H18" s="223"/>
+      <c r="I18" s="222"/>
+      <c r="J18" s="222"/>
+      <c r="K18" s="227"/>
+      <c r="L18" s="222"/>
     </row>
     <row r="19" spans="1:21" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -19460,17 +19460,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="190" priority="8" operator="equal">
@@ -19957,38 +19957,38 @@
       </c>
     </row>
     <row r="8" spans="1:21" ht="28.8">
-      <c r="A8" s="222" t="s">
+      <c r="A8" s="224" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="227" t="s">
+      <c r="B8" s="225" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="222" t="s">
+      <c r="C8" s="224" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="234" t="s">
+      <c r="D8" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E8" s="224" t="s">
+      <c r="E8" s="226" t="s">
         <v>296</v>
       </c>
-      <c r="F8" s="221" t="s">
+      <c r="F8" s="223" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="221" t="s">
+      <c r="G8" s="223" t="s">
         <v>99</v>
       </c>
-      <c r="H8" s="221" t="s">
+      <c r="H8" s="223" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="225" t="s">
+      <c r="I8" s="222" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="225" t="s">
+      <c r="J8" s="222" t="s">
         <v>30</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="225"/>
+      <c r="L8" s="222"/>
       <c r="M8" s="32" t="s">
         <v>703</v>
       </c>
@@ -20006,20 +20006,20 @@
       </c>
     </row>
     <row r="9" spans="1:21" ht="28.8">
-      <c r="A9" s="222"/>
-      <c r="B9" s="227"/>
-      <c r="C9" s="222"/>
-      <c r="D9" s="234" t="s">
+      <c r="A9" s="224"/>
+      <c r="B9" s="225"/>
+      <c r="C9" s="224"/>
+      <c r="D9" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E9" s="224"/>
-      <c r="F9" s="221"/>
-      <c r="G9" s="221"/>
-      <c r="H9" s="221"/>
-      <c r="I9" s="225"/>
-      <c r="J9" s="225"/>
+      <c r="E9" s="226"/>
+      <c r="F9" s="223"/>
+      <c r="G9" s="223"/>
+      <c r="H9" s="223"/>
+      <c r="I9" s="222"/>
+      <c r="J9" s="222"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="225"/>
+      <c r="L9" s="222"/>
       <c r="M9" s="32" t="s">
         <v>782</v>
       </c>
@@ -20028,20 +20028,20 @@
       </c>
     </row>
     <row r="10" spans="1:21" ht="28.8">
-      <c r="A10" s="222"/>
-      <c r="B10" s="227"/>
-      <c r="C10" s="222"/>
-      <c r="D10" s="234" t="s">
+      <c r="A10" s="224"/>
+      <c r="B10" s="225"/>
+      <c r="C10" s="224"/>
+      <c r="D10" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E10" s="224"/>
-      <c r="F10" s="221"/>
-      <c r="G10" s="221"/>
-      <c r="H10" s="221"/>
-      <c r="I10" s="225"/>
-      <c r="J10" s="225"/>
+      <c r="E10" s="226"/>
+      <c r="F10" s="223"/>
+      <c r="G10" s="223"/>
+      <c r="H10" s="223"/>
+      <c r="I10" s="222"/>
+      <c r="J10" s="222"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="225"/>
+      <c r="L10" s="222"/>
       <c r="M10" s="32" t="s">
         <v>782</v>
       </c>
@@ -20050,20 +20050,20 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="222"/>
-      <c r="B11" s="227"/>
-      <c r="C11" s="222"/>
-      <c r="D11" s="234" t="s">
+      <c r="A11" s="224"/>
+      <c r="B11" s="225"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E11" s="224"/>
-      <c r="F11" s="221"/>
-      <c r="G11" s="221"/>
-      <c r="H11" s="221"/>
-      <c r="I11" s="225"/>
-      <c r="J11" s="225"/>
+      <c r="E11" s="226"/>
+      <c r="F11" s="223"/>
+      <c r="G11" s="223"/>
+      <c r="H11" s="223"/>
+      <c r="I11" s="222"/>
+      <c r="J11" s="222"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="225"/>
+      <c r="L11" s="222"/>
       <c r="M11" s="32" t="s">
         <v>782</v>
       </c>
@@ -20072,20 +20072,20 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="222"/>
-      <c r="B12" s="227"/>
-      <c r="C12" s="222"/>
-      <c r="D12" s="234" t="s">
+      <c r="A12" s="224"/>
+      <c r="B12" s="225"/>
+      <c r="C12" s="224"/>
+      <c r="D12" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E12" s="224"/>
-      <c r="F12" s="221"/>
-      <c r="G12" s="221"/>
-      <c r="H12" s="221"/>
-      <c r="I12" s="225"/>
-      <c r="J12" s="225"/>
+      <c r="E12" s="226"/>
+      <c r="F12" s="223"/>
+      <c r="G12" s="223"/>
+      <c r="H12" s="223"/>
+      <c r="I12" s="222"/>
+      <c r="J12" s="222"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="225"/>
+      <c r="L12" s="222"/>
       <c r="M12" s="32" t="s">
         <v>782</v>
       </c>
@@ -23291,6 +23291,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -23533,28 +23554,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
+    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23571,23 +23590,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
-    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update metadata to Health-RI v2.0.3 (#12)
* Update metadata to Health-RI v2.0.3

Upgrade to Health-RI v2.0.3 specification and regenerate property documentation.

Changes include:
- Updated Excel metadata specification from v2.0.2 to v2.0.3
- Corrected type definitions (e.g., xsd:string → rdfs:Literal)
- Updated cardinalities for dataset requirement (0..n → 1..n)
- Enhanced creator and contact point descriptions with clarifications
- Standardized contact point language across all properties
- Fixed formatting and URL protocols
- Improved documentation with additional guidance and examples

* Delete src/excel/~$HealthRI_v2.0.2.xlsx

deleted temp file

* Update UML class diagram description to 2.0.3

Bump the UML Class Diagram version from v2.0.2 to v2.0.3 in the introduction chapter.

* removal of the \n error

the removal of '\n' in the documentation is done manually for now, but this needs a fix for the complete automation from excel again
</commit_message>
<xml_diff>
--- a/src/excel/HealthRI_v2.0.2.xlsx
+++ b/src/excel/HealthRI_v2.0.2.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D452F6-957B-427A-8247-D60DE431818C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11604" windowHeight="13776" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -4101,32 +4101,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -4140,8 +4137,11 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -9796,40 +9796,40 @@
       </c>
     </row>
     <row r="6" spans="1:21" ht="28.8">
-      <c r="A6" s="231" t="s">
+      <c r="A6" s="230" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="232" t="s">
+      <c r="B6" s="231" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="231" t="s">
+      <c r="C6" s="230" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="234" t="s">
+      <c r="D6" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E6" s="233" t="s">
+      <c r="E6" s="232" t="s">
         <v>98</v>
       </c>
-      <c r="F6" s="230" t="s">
+      <c r="F6" s="229" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="230" t="s">
+      <c r="G6" s="229" t="s">
         <v>99</v>
       </c>
-      <c r="H6" s="230" t="s">
+      <c r="H6" s="229" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="228" t="s">
+      <c r="I6" s="233" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="225" t="s">
+      <c r="J6" s="222" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="229" t="s">
+      <c r="K6" s="234" t="s">
         <v>456</v>
       </c>
-      <c r="L6" s="228"/>
+      <c r="L6" s="233"/>
       <c r="M6" s="32" t="s">
         <v>703</v>
       </c>
@@ -9847,68 +9847,68 @@
       </c>
     </row>
     <row r="7" spans="1:21" ht="28.8">
-      <c r="A7" s="231"/>
-      <c r="B7" s="232"/>
-      <c r="C7" s="231"/>
-      <c r="D7" s="234" t="s">
+      <c r="A7" s="230"/>
+      <c r="B7" s="231"/>
+      <c r="C7" s="230"/>
+      <c r="D7" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E7" s="233"/>
-      <c r="F7" s="230"/>
-      <c r="G7" s="230"/>
-      <c r="H7" s="230"/>
-      <c r="I7" s="228"/>
-      <c r="J7" s="225"/>
-      <c r="K7" s="229"/>
-      <c r="L7" s="228"/>
+      <c r="E7" s="232"/>
+      <c r="F7" s="229"/>
+      <c r="G7" s="229"/>
+      <c r="H7" s="229"/>
+      <c r="I7" s="233"/>
+      <c r="J7" s="222"/>
+      <c r="K7" s="234"/>
+      <c r="L7" s="233"/>
     </row>
     <row r="8" spans="1:21" ht="28.8">
-      <c r="A8" s="231"/>
-      <c r="B8" s="232"/>
-      <c r="C8" s="231"/>
-      <c r="D8" s="234" t="s">
+      <c r="A8" s="230"/>
+      <c r="B8" s="231"/>
+      <c r="C8" s="230"/>
+      <c r="D8" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E8" s="233"/>
-      <c r="F8" s="230"/>
-      <c r="G8" s="230"/>
-      <c r="H8" s="230"/>
-      <c r="I8" s="228"/>
-      <c r="J8" s="225"/>
-      <c r="K8" s="229"/>
-      <c r="L8" s="228"/>
+      <c r="E8" s="232"/>
+      <c r="F8" s="229"/>
+      <c r="G8" s="229"/>
+      <c r="H8" s="229"/>
+      <c r="I8" s="233"/>
+      <c r="J8" s="222"/>
+      <c r="K8" s="234"/>
+      <c r="L8" s="233"/>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="231"/>
-      <c r="B9" s="232"/>
-      <c r="C9" s="231"/>
-      <c r="D9" s="234" t="s">
+      <c r="A9" s="230"/>
+      <c r="B9" s="231"/>
+      <c r="C9" s="230"/>
+      <c r="D9" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E9" s="233"/>
-      <c r="F9" s="230"/>
-      <c r="G9" s="230"/>
-      <c r="H9" s="230"/>
-      <c r="I9" s="228"/>
-      <c r="J9" s="225"/>
-      <c r="K9" s="229"/>
-      <c r="L9" s="228"/>
+      <c r="E9" s="232"/>
+      <c r="F9" s="229"/>
+      <c r="G9" s="229"/>
+      <c r="H9" s="229"/>
+      <c r="I9" s="233"/>
+      <c r="J9" s="222"/>
+      <c r="K9" s="234"/>
+      <c r="L9" s="233"/>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="231"/>
-      <c r="B10" s="232"/>
-      <c r="C10" s="231"/>
-      <c r="D10" s="234" t="s">
+      <c r="A10" s="230"/>
+      <c r="B10" s="231"/>
+      <c r="C10" s="230"/>
+      <c r="D10" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E10" s="233"/>
-      <c r="F10" s="230"/>
-      <c r="G10" s="230"/>
-      <c r="H10" s="230"/>
-      <c r="I10" s="228"/>
-      <c r="J10" s="225"/>
-      <c r="K10" s="229"/>
-      <c r="L10" s="228"/>
+      <c r="E10" s="232"/>
+      <c r="F10" s="229"/>
+      <c r="G10" s="229"/>
+      <c r="H10" s="229"/>
+      <c r="I10" s="233"/>
+      <c r="J10" s="222"/>
+      <c r="K10" s="234"/>
+      <c r="L10" s="233"/>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="121" t="s">
@@ -10303,17 +10303,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -11281,7 +11281,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="57.6">
+    <row r="18" spans="1:21" ht="43.2">
       <c r="A18" s="121" t="s">
         <v>155</v>
       </c>
@@ -16172,74 +16172,74 @@
       <c r="L13" s="129"/>
     </row>
     <row r="14" spans="1:20">
-      <c r="A14" s="222"/>
-      <c r="B14" s="223"/>
-      <c r="C14" s="222"/>
+      <c r="A14" s="224"/>
+      <c r="B14" s="228"/>
+      <c r="C14" s="224"/>
       <c r="D14" s="151"/>
-      <c r="E14" s="224"/>
-      <c r="F14" s="221"/>
-      <c r="G14" s="221"/>
-      <c r="H14" s="221"/>
-      <c r="I14" s="225"/>
-      <c r="J14" s="225"/>
-      <c r="K14" s="226"/>
-      <c r="L14" s="225"/>
+      <c r="E14" s="226"/>
+      <c r="F14" s="223"/>
+      <c r="G14" s="223"/>
+      <c r="H14" s="223"/>
+      <c r="I14" s="222"/>
+      <c r="J14" s="222"/>
+      <c r="K14" s="227"/>
+      <c r="L14" s="222"/>
     </row>
     <row r="15" spans="1:20">
-      <c r="A15" s="222"/>
-      <c r="B15" s="223"/>
-      <c r="C15" s="222"/>
+      <c r="A15" s="224"/>
+      <c r="B15" s="228"/>
+      <c r="C15" s="224"/>
       <c r="D15" s="152"/>
-      <c r="E15" s="224"/>
-      <c r="F15" s="221"/>
-      <c r="G15" s="221"/>
-      <c r="H15" s="221"/>
-      <c r="I15" s="225"/>
-      <c r="J15" s="225"/>
-      <c r="K15" s="226"/>
-      <c r="L15" s="225"/>
+      <c r="E15" s="226"/>
+      <c r="F15" s="223"/>
+      <c r="G15" s="223"/>
+      <c r="H15" s="223"/>
+      <c r="I15" s="222"/>
+      <c r="J15" s="222"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="222"/>
     </row>
     <row r="16" spans="1:20">
-      <c r="A16" s="222"/>
-      <c r="B16" s="223"/>
-      <c r="C16" s="222"/>
+      <c r="A16" s="224"/>
+      <c r="B16" s="228"/>
+      <c r="C16" s="224"/>
       <c r="D16" s="152"/>
-      <c r="E16" s="224"/>
-      <c r="F16" s="221"/>
-      <c r="G16" s="221"/>
-      <c r="H16" s="221"/>
-      <c r="I16" s="225"/>
-      <c r="J16" s="225"/>
-      <c r="K16" s="226"/>
-      <c r="L16" s="225"/>
+      <c r="E16" s="226"/>
+      <c r="F16" s="223"/>
+      <c r="G16" s="223"/>
+      <c r="H16" s="223"/>
+      <c r="I16" s="222"/>
+      <c r="J16" s="222"/>
+      <c r="K16" s="227"/>
+      <c r="L16" s="222"/>
     </row>
     <row r="17" spans="1:12">
-      <c r="A17" s="222"/>
-      <c r="B17" s="223"/>
-      <c r="C17" s="222"/>
+      <c r="A17" s="224"/>
+      <c r="B17" s="228"/>
+      <c r="C17" s="224"/>
       <c r="D17" s="152"/>
-      <c r="E17" s="224"/>
-      <c r="F17" s="221"/>
-      <c r="G17" s="221"/>
-      <c r="H17" s="221"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="225"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="225"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="223"/>
+      <c r="G17" s="223"/>
+      <c r="H17" s="223"/>
+      <c r="I17" s="222"/>
+      <c r="J17" s="222"/>
+      <c r="K17" s="227"/>
+      <c r="L17" s="222"/>
     </row>
     <row r="18" spans="1:12">
-      <c r="A18" s="222"/>
-      <c r="B18" s="223"/>
-      <c r="C18" s="222"/>
+      <c r="A18" s="224"/>
+      <c r="B18" s="228"/>
+      <c r="C18" s="224"/>
       <c r="D18" s="152"/>
-      <c r="E18" s="224"/>
-      <c r="F18" s="221"/>
-      <c r="G18" s="221"/>
-      <c r="H18" s="221"/>
-      <c r="I18" s="225"/>
-      <c r="J18" s="225"/>
-      <c r="K18" s="226"/>
-      <c r="L18" s="225"/>
+      <c r="E18" s="226"/>
+      <c r="F18" s="223"/>
+      <c r="G18" s="223"/>
+      <c r="H18" s="223"/>
+      <c r="I18" s="222"/>
+      <c r="J18" s="222"/>
+      <c r="K18" s="227"/>
+      <c r="L18" s="222"/>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="125"/>
@@ -16747,17 +16747,17 @@
   </sheetData>
   <autoFilter ref="A1:J53" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="11">
-    <mergeCell ref="H14:H18"/>
-    <mergeCell ref="I14:I18"/>
-    <mergeCell ref="J14:J18"/>
-    <mergeCell ref="K14:K18"/>
-    <mergeCell ref="L14:L18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="A14:A18"/>
     <mergeCell ref="B14:B18"/>
     <mergeCell ref="C14:C18"/>
     <mergeCell ref="E14:E18"/>
     <mergeCell ref="F14:F18"/>
+    <mergeCell ref="H14:H18"/>
+    <mergeCell ref="I14:I18"/>
+    <mergeCell ref="J14:J18"/>
+    <mergeCell ref="K14:K18"/>
+    <mergeCell ref="L14:L18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="204" priority="8" operator="equal">
@@ -17555,38 +17555,38 @@
       </c>
     </row>
     <row r="14" spans="1:21" ht="43.2">
-      <c r="A14" s="222" t="s">
+      <c r="A14" s="224" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="223" t="s">
+      <c r="B14" s="228" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="222" t="s">
+      <c r="C14" s="224" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="234" t="s">
+      <c r="D14" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E14" s="224" t="s">
+      <c r="E14" s="226" t="s">
         <v>98</v>
       </c>
-      <c r="F14" s="221" t="s">
+      <c r="F14" s="223" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="221" t="s">
+      <c r="G14" s="223" t="s">
         <v>99</v>
       </c>
-      <c r="H14" s="221" t="s">
+      <c r="H14" s="223" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="225" t="s">
+      <c r="I14" s="222" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="225" t="s">
+      <c r="J14" s="222" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="226"/>
-      <c r="L14" s="225"/>
+      <c r="K14" s="227"/>
+      <c r="L14" s="222"/>
       <c r="M14" s="32" t="s">
         <v>703</v>
       </c>
@@ -17604,68 +17604,68 @@
       </c>
     </row>
     <row r="15" spans="1:21" ht="43.2">
-      <c r="A15" s="222"/>
-      <c r="B15" s="223"/>
-      <c r="C15" s="222"/>
-      <c r="D15" s="234" t="s">
+      <c r="A15" s="224"/>
+      <c r="B15" s="228"/>
+      <c r="C15" s="224"/>
+      <c r="D15" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E15" s="224"/>
-      <c r="F15" s="221"/>
-      <c r="G15" s="221"/>
-      <c r="H15" s="221"/>
-      <c r="I15" s="225"/>
-      <c r="J15" s="225"/>
-      <c r="K15" s="226"/>
-      <c r="L15" s="225"/>
+      <c r="E15" s="226"/>
+      <c r="F15" s="223"/>
+      <c r="G15" s="223"/>
+      <c r="H15" s="223"/>
+      <c r="I15" s="222"/>
+      <c r="J15" s="222"/>
+      <c r="K15" s="227"/>
+      <c r="L15" s="222"/>
     </row>
     <row r="16" spans="1:21" ht="28.8">
-      <c r="A16" s="222"/>
-      <c r="B16" s="223"/>
-      <c r="C16" s="222"/>
-      <c r="D16" s="234" t="s">
+      <c r="A16" s="224"/>
+      <c r="B16" s="228"/>
+      <c r="C16" s="224"/>
+      <c r="D16" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E16" s="224"/>
-      <c r="F16" s="221"/>
-      <c r="G16" s="221"/>
-      <c r="H16" s="221"/>
-      <c r="I16" s="225"/>
-      <c r="J16" s="225"/>
-      <c r="K16" s="226"/>
-      <c r="L16" s="225"/>
+      <c r="E16" s="226"/>
+      <c r="F16" s="223"/>
+      <c r="G16" s="223"/>
+      <c r="H16" s="223"/>
+      <c r="I16" s="222"/>
+      <c r="J16" s="222"/>
+      <c r="K16" s="227"/>
+      <c r="L16" s="222"/>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="222"/>
-      <c r="B17" s="223"/>
-      <c r="C17" s="222"/>
-      <c r="D17" s="234" t="s">
+      <c r="A17" s="224"/>
+      <c r="B17" s="228"/>
+      <c r="C17" s="224"/>
+      <c r="D17" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E17" s="224"/>
-      <c r="F17" s="221"/>
-      <c r="G17" s="221"/>
-      <c r="H17" s="221"/>
-      <c r="I17" s="225"/>
-      <c r="J17" s="225"/>
-      <c r="K17" s="226"/>
-      <c r="L17" s="225"/>
+      <c r="E17" s="226"/>
+      <c r="F17" s="223"/>
+      <c r="G17" s="223"/>
+      <c r="H17" s="223"/>
+      <c r="I17" s="222"/>
+      <c r="J17" s="222"/>
+      <c r="K17" s="227"/>
+      <c r="L17" s="222"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="222"/>
-      <c r="B18" s="223"/>
-      <c r="C18" s="222"/>
-      <c r="D18" s="234" t="s">
+      <c r="A18" s="224"/>
+      <c r="B18" s="228"/>
+      <c r="C18" s="224"/>
+      <c r="D18" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E18" s="224"/>
-      <c r="F18" s="221"/>
-      <c r="G18" s="221"/>
-      <c r="H18" s="221"/>
-      <c r="I18" s="225"/>
-      <c r="J18" s="225"/>
-      <c r="K18" s="226"/>
-      <c r="L18" s="225"/>
+      <c r="E18" s="226"/>
+      <c r="F18" s="223"/>
+      <c r="G18" s="223"/>
+      <c r="H18" s="223"/>
+      <c r="I18" s="222"/>
+      <c r="J18" s="222"/>
+      <c r="K18" s="227"/>
+      <c r="L18" s="222"/>
     </row>
     <row r="19" spans="1:21" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -19460,17 +19460,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="190" priority="8" operator="equal">
@@ -19957,38 +19957,38 @@
       </c>
     </row>
     <row r="8" spans="1:21" ht="28.8">
-      <c r="A8" s="222" t="s">
+      <c r="A8" s="224" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="227" t="s">
+      <c r="B8" s="225" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="222" t="s">
+      <c r="C8" s="224" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="234" t="s">
+      <c r="D8" s="221" t="s">
         <v>894</v>
       </c>
-      <c r="E8" s="224" t="s">
+      <c r="E8" s="226" t="s">
         <v>296</v>
       </c>
-      <c r="F8" s="221" t="s">
+      <c r="F8" s="223" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="221" t="s">
+      <c r="G8" s="223" t="s">
         <v>99</v>
       </c>
-      <c r="H8" s="221" t="s">
+      <c r="H8" s="223" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="225" t="s">
+      <c r="I8" s="222" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="225" t="s">
+      <c r="J8" s="222" t="s">
         <v>30</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="225"/>
+      <c r="L8" s="222"/>
       <c r="M8" s="32" t="s">
         <v>703</v>
       </c>
@@ -20006,20 +20006,20 @@
       </c>
     </row>
     <row r="9" spans="1:21" ht="28.8">
-      <c r="A9" s="222"/>
-      <c r="B9" s="227"/>
-      <c r="C9" s="222"/>
-      <c r="D9" s="234" t="s">
+      <c r="A9" s="224"/>
+      <c r="B9" s="225"/>
+      <c r="C9" s="224"/>
+      <c r="D9" s="221" t="s">
         <v>895</v>
       </c>
-      <c r="E9" s="224"/>
-      <c r="F9" s="221"/>
-      <c r="G9" s="221"/>
-      <c r="H9" s="221"/>
-      <c r="I9" s="225"/>
-      <c r="J9" s="225"/>
+      <c r="E9" s="226"/>
+      <c r="F9" s="223"/>
+      <c r="G9" s="223"/>
+      <c r="H9" s="223"/>
+      <c r="I9" s="222"/>
+      <c r="J9" s="222"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="225"/>
+      <c r="L9" s="222"/>
       <c r="M9" s="32" t="s">
         <v>782</v>
       </c>
@@ -20028,20 +20028,20 @@
       </c>
     </row>
     <row r="10" spans="1:21" ht="28.8">
-      <c r="A10" s="222"/>
-      <c r="B10" s="227"/>
-      <c r="C10" s="222"/>
-      <c r="D10" s="234" t="s">
+      <c r="A10" s="224"/>
+      <c r="B10" s="225"/>
+      <c r="C10" s="224"/>
+      <c r="D10" s="221" t="s">
         <v>896</v>
       </c>
-      <c r="E10" s="224"/>
-      <c r="F10" s="221"/>
-      <c r="G10" s="221"/>
-      <c r="H10" s="221"/>
-      <c r="I10" s="225"/>
-      <c r="J10" s="225"/>
+      <c r="E10" s="226"/>
+      <c r="F10" s="223"/>
+      <c r="G10" s="223"/>
+      <c r="H10" s="223"/>
+      <c r="I10" s="222"/>
+      <c r="J10" s="222"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="225"/>
+      <c r="L10" s="222"/>
       <c r="M10" s="32" t="s">
         <v>782</v>
       </c>
@@ -20050,20 +20050,20 @@
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="222"/>
-      <c r="B11" s="227"/>
-      <c r="C11" s="222"/>
-      <c r="D11" s="234" t="s">
+      <c r="A11" s="224"/>
+      <c r="B11" s="225"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="221" t="s">
         <v>897</v>
       </c>
-      <c r="E11" s="224"/>
-      <c r="F11" s="221"/>
-      <c r="G11" s="221"/>
-      <c r="H11" s="221"/>
-      <c r="I11" s="225"/>
-      <c r="J11" s="225"/>
+      <c r="E11" s="226"/>
+      <c r="F11" s="223"/>
+      <c r="G11" s="223"/>
+      <c r="H11" s="223"/>
+      <c r="I11" s="222"/>
+      <c r="J11" s="222"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="225"/>
+      <c r="L11" s="222"/>
       <c r="M11" s="32" t="s">
         <v>782</v>
       </c>
@@ -20072,20 +20072,20 @@
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="222"/>
-      <c r="B12" s="227"/>
-      <c r="C12" s="222"/>
-      <c r="D12" s="234" t="s">
+      <c r="A12" s="224"/>
+      <c r="B12" s="225"/>
+      <c r="C12" s="224"/>
+      <c r="D12" s="221" t="s">
         <v>898</v>
       </c>
-      <c r="E12" s="224"/>
-      <c r="F12" s="221"/>
-      <c r="G12" s="221"/>
-      <c r="H12" s="221"/>
-      <c r="I12" s="225"/>
-      <c r="J12" s="225"/>
+      <c r="E12" s="226"/>
+      <c r="F12" s="223"/>
+      <c r="G12" s="223"/>
+      <c r="H12" s="223"/>
+      <c r="I12" s="222"/>
+      <c r="J12" s="222"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="225"/>
+      <c r="L12" s="222"/>
       <c r="M12" s="32" t="s">
         <v>782</v>
       </c>
@@ -23291,6 +23291,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -23533,28 +23554,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Status xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">Draft</Status>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cfc87205-1831-4b6c-a7b4-76d40079a43e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="221af607-abea-4d5e-830c-567dcc03c0ec" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
+    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23571,23 +23590,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
-    <ds:schemaRef ds:uri="221af607-abea-4d5e-830c-567dcc03c0ec"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>